<commit_message>
Admin: edit data/team.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/team.xlsx
+++ b/data/team.xlsx
@@ -489,7 +489,7 @@
         <v>Priyanka Sasane</v>
       </c>
       <c r="B6" t="str">
-        <v>Acting Secretory</v>
+        <v>Acting Secretary</v>
       </c>
       <c r="C6" t="str">
         <v>Executive Members</v>
@@ -588,7 +588,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Abhai Naik</v>
+        <v>Abhay Naik</v>
       </c>
       <c r="B12" t="str">
         <v>Process &amp; Marketing Head</v>

</xml_diff>